<commit_message>
Estadisticos Final 10 Listados
</commit_message>
<xml_diff>
--- a/Calificaciones20241.xlsx
+++ b/Calificaciones20241.xlsx
@@ -48330,7 +48330,7 @@
         <v>10</v>
       </c>
       <c r="V4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W4">
         <v>8</v>
@@ -48419,7 +48419,7 @@
         <v>6</v>
       </c>
       <c r="V5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W5">
         <v>5</v>
@@ -48440,7 +48440,7 @@
         <v>7</v>
       </c>
       <c r="AC5">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:29">
@@ -48508,7 +48508,7 @@
         <v>8</v>
       </c>
       <c r="V6">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W6">
         <v>5</v>
@@ -48529,7 +48529,7 @@
         <v>9</v>
       </c>
       <c r="AC6">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:29">
@@ -48597,7 +48597,7 @@
         <v>9</v>
       </c>
       <c r="V7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W7">
         <v>9</v>
@@ -48686,7 +48686,7 @@
         <v>6</v>
       </c>
       <c r="V8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W8">
         <v>5</v>
@@ -48775,7 +48775,7 @@
         <v>9</v>
       </c>
       <c r="V9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W9">
         <v>7</v>
@@ -48864,7 +48864,7 @@
         <v>6</v>
       </c>
       <c r="V10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W10">
         <v>5</v>
@@ -48953,7 +48953,7 @@
         <v>8</v>
       </c>
       <c r="V11">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W11">
         <v>7</v>
@@ -49042,7 +49042,7 @@
         <v>6</v>
       </c>
       <c r="V12">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W12">
         <v>5</v>
@@ -49131,7 +49131,7 @@
         <v>8</v>
       </c>
       <c r="V13">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W13">
         <v>5</v>
@@ -49220,7 +49220,7 @@
         <v>7</v>
       </c>
       <c r="V14">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W14">
         <v>6</v>
@@ -49309,7 +49309,7 @@
         <v>10</v>
       </c>
       <c r="V15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W15">
         <v>7</v>
@@ -49330,7 +49330,7 @@
         <v>10</v>
       </c>
       <c r="AC15">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:29">
@@ -49398,7 +49398,7 @@
         <v>8</v>
       </c>
       <c r="V16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W16">
         <v>5</v>
@@ -49419,7 +49419,7 @@
         <v>9</v>
       </c>
       <c r="AC16">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:29">
@@ -49487,7 +49487,7 @@
         <v>7</v>
       </c>
       <c r="V17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W17">
         <v>5</v>
@@ -49576,7 +49576,7 @@
         <v>6</v>
       </c>
       <c r="V18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W18">
         <v>5</v>
@@ -49665,7 +49665,7 @@
         <v>6</v>
       </c>
       <c r="V19">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W19">
         <v>5</v>
@@ -49754,7 +49754,7 @@
         <v>7</v>
       </c>
       <c r="V20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W20">
         <v>5</v>
@@ -49843,7 +49843,7 @@
         <v>8</v>
       </c>
       <c r="V21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W21">
         <v>6</v>
@@ -49864,7 +49864,7 @@
         <v>9</v>
       </c>
       <c r="AC21">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:29">
@@ -49932,7 +49932,7 @@
         <v>8</v>
       </c>
       <c r="V22">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W22">
         <v>7</v>
@@ -50021,7 +50021,7 @@
         <v>8</v>
       </c>
       <c r="V23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W23">
         <v>5</v>
@@ -50110,7 +50110,7 @@
         <v>7</v>
       </c>
       <c r="V24">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W24">
         <v>8</v>
@@ -50131,7 +50131,7 @@
         <v>7</v>
       </c>
       <c r="AC24">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:29">
@@ -50199,7 +50199,7 @@
         <v>9</v>
       </c>
       <c r="V25">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W25">
         <v>9</v>
@@ -50220,7 +50220,7 @@
         <v>9</v>
       </c>
       <c r="AC25">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26" spans="1:29">
@@ -50288,7 +50288,7 @@
         <v>9</v>
       </c>
       <c r="V26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W26">
         <v>7</v>
@@ -52372,7 +52372,7 @@
         <v>9</v>
       </c>
       <c r="V4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W4">
         <v>8</v>
@@ -52393,7 +52393,7 @@
         <v>8</v>
       </c>
       <c r="AC4">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:29">
@@ -52490,7 +52490,7 @@
         <v>7</v>
       </c>
       <c r="V6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W6">
         <v>9</v>
@@ -52579,7 +52579,7 @@
         <v>7</v>
       </c>
       <c r="V7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W7">
         <v>7</v>
@@ -52668,7 +52668,7 @@
         <v>8</v>
       </c>
       <c r="V8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W8">
         <v>9</v>
@@ -52689,7 +52689,7 @@
         <v>8</v>
       </c>
       <c r="AC8">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:29">
@@ -52757,7 +52757,7 @@
         <v>7</v>
       </c>
       <c r="V9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W9">
         <v>7</v>
@@ -52846,7 +52846,7 @@
         <v>7</v>
       </c>
       <c r="V10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W10">
         <v>8</v>
@@ -52867,7 +52867,7 @@
         <v>6</v>
       </c>
       <c r="AC10">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:29">
@@ -52935,7 +52935,7 @@
         <v>7</v>
       </c>
       <c r="V11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W11">
         <v>7</v>
@@ -53024,7 +53024,7 @@
         <v>8</v>
       </c>
       <c r="V12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W12">
         <v>9</v>
@@ -53045,7 +53045,7 @@
         <v>7</v>
       </c>
       <c r="AC12">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:29">
@@ -53113,7 +53113,7 @@
         <v>6</v>
       </c>
       <c r="V13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W13">
         <v>8</v>
@@ -53202,7 +53202,7 @@
         <v>7</v>
       </c>
       <c r="V14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W14">
         <v>8</v>
@@ -53291,7 +53291,7 @@
         <v>7</v>
       </c>
       <c r="V15">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W15">
         <v>6</v>
@@ -53312,7 +53312,7 @@
         <v>6</v>
       </c>
       <c r="AC15">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:29">
@@ -53380,7 +53380,7 @@
         <v>9</v>
       </c>
       <c r="V16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W16">
         <v>9</v>
@@ -53469,7 +53469,7 @@
         <v>7</v>
       </c>
       <c r="V17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W17">
         <v>8</v>
@@ -53490,7 +53490,7 @@
         <v>7</v>
       </c>
       <c r="AC17">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:29">
@@ -53558,7 +53558,7 @@
         <v>5</v>
       </c>
       <c r="V18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W18">
         <v>8</v>
@@ -53647,7 +53647,7 @@
         <v>8</v>
       </c>
       <c r="V19">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W19">
         <v>8</v>
@@ -53668,7 +53668,7 @@
         <v>7</v>
       </c>
       <c r="AC19">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:29">
@@ -53736,7 +53736,7 @@
         <v>7</v>
       </c>
       <c r="V20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W20">
         <v>7</v>
@@ -53825,7 +53825,7 @@
         <v>8</v>
       </c>
       <c r="V21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W21">
         <v>7</v>
@@ -53914,7 +53914,7 @@
         <v>8</v>
       </c>
       <c r="V22">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W22">
         <v>7</v>
@@ -54003,7 +54003,7 @@
         <v>5</v>
       </c>
       <c r="V23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W23">
         <v>5</v>
@@ -54092,7 +54092,7 @@
         <v>8</v>
       </c>
       <c r="V24">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W24">
         <v>8</v>
@@ -54181,7 +54181,7 @@
         <v>8</v>
       </c>
       <c r="V25">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W25">
         <v>9</v>
@@ -54202,7 +54202,7 @@
         <v>8</v>
       </c>
       <c r="AC25">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>